<commit_message>
feat: implement canonical tree normalization engine to enforce consistent X-Y-Z-W-Q hierarchy and enable automatic node grouping
</commit_message>
<xml_diff>
--- a/bug rotacao.xlsx
+++ b/bug rotacao.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>ID</t>
   </si>
@@ -38,7 +38,37 @@
     <t>Largura</t>
   </si>
   <si>
-    <t>teste</t>
+    <t>a</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>e</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
+    <t>j</t>
+  </si>
+  <si>
+    <t>k</t>
   </si>
 </sst>
 </file>
@@ -371,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.85546875" bestFit="1" customWidth="1"/>
@@ -399,7 +429,7 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C2">
         <v>917</v>
@@ -410,15 +440,141 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3">
+        <v>917</v>
+      </c>
+      <c r="D3">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>917</v>
+      </c>
+      <c r="D4">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>917</v>
+      </c>
+      <c r="D5">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>917</v>
+      </c>
+      <c r="D6">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>917</v>
+      </c>
+      <c r="D7">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>917</v>
+      </c>
+      <c r="D8">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>917</v>
+      </c>
+      <c r="D9">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>917</v>
+      </c>
+      <c r="D10">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>917</v>
+      </c>
+      <c r="D11">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
         <v>459</v>
       </c>
-      <c r="D3">
+      <c r="D12">
         <v>1000</v>
       </c>
     </row>

</xml_diff>